<commit_message>
Add Excel sync automation workflow
</commit_message>
<xml_diff>
--- a/output/Job_Dashboard.xlsx
+++ b/output/Job_Dashboard.xlsx
@@ -4541,7 +4541,17 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>To Review</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>0806</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>A1 TEST</t>
         </is>
       </c>
     </row>
@@ -8132,7 +8142,6 @@
       <c r="F10" t="n">
         <v>28</v>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Partial</t>

</xml_diff>

<commit_message>
Auto update Job Dashboard
</commit_message>
<xml_diff>
--- a/output/Job_Dashboard.xlsx
+++ b/output/Job_Dashboard.xlsx
@@ -2896,7 +2896,13 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>To Review</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>test</t>
         </is>
       </c>
     </row>
@@ -8624,7 +8630,6 @@
       <c r="F11" t="n">
         <v>31</v>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Partial</t>

</xml_diff>